<commit_message>
chore: preparar repositório para produção
- Remove PDFs e documento de análise acadêmica desnecessários
- Remove código morto (RegistroService + RegistroDiario) nunca usado no app
- Renova README.md com visão completa: funcionalidades, setup Docker/sem Docker, env vars, arquitetura e troubleshooting
- Melhora ARQUITETURA.md: adiciona AlunoTabNotifier (pausa de vídeo), chat local e re-export de tema
- Melhora COMO-TESTAR.md: documenta pausa e retomada de vídeo por aba
- Adiciona casos de teste 4.9, 5.10–5.12 no QA-TESTES.md e QA-TESTES.xlsx (video pause/resume, dropdown crash)
- Corrige prefer_const nos testes unitários (flutter analyze: 0 issues)
</commit_message>
<xml_diff>
--- a/docs/QA-TESTES.xlsx
+++ b/docs/QA-TESTES.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1498,314 +1498,314 @@
       <c r="G34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Criar/Editar Treino</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Remover aluno e voltar a criacao de treino (anti-crash dropdown)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Aluno removido nao aparece no dropdown; sem crash de item invalido selecionado</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Critico</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Ver treinos do dia</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Lista por dia com series/reps/carga</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Video do exercicio</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Thumbnail aparece; toca e reproduz</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Descricao Como executar</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Expande/recolhe e mostra o texto</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Marcar exercicio como feito</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Vira Concluido; entra na Atividade Recente</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Conclusao persiste apos reabrir</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Exercicio/treino continua concluido</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>5.6</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Desmarcar</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Volta a pendente; persiste apos reabrir</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>5.7</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Marcar com peso (1,5 e 1.5)</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Registra peso corretamente</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>5.8</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Concluir treino do dia</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Vira selo Treino concluido; persiste</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>5.9</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Treinos Aluno</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Conclusao por usuario</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>Concluido do A nao aparece para o B</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>6.1</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Offline-First</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Abrir treinos online e depois offline</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Treinos continuam visiveis (cache)</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Critico</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.10</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Offline-First</t>
+          <t>Treinos Aluno</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Abrir offline sem cache (1a vez)</t>
+          <t>Video pausa ao trocar de aba</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Mensagem amigavel; sem crash/logout</t>
+          <t>Reproduzir video -&gt; trocar para outra aba -&gt; audio/video para; sem crash</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -1813,71 +1813,71 @@
           <t>Critico</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>6.3</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Offline-First</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Backend desligado</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Erro com Tentar novamente; sem logout</t>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>5.11</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Treinos Aluno</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Video retoma da posicao salva</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Apos pausa (5.10), voltar a aba Treinos -&gt; play -&gt; video comeca no ponto em que parou</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Critico</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>5.12</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Offline-First</t>
+          <t>Treinos Aluno</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Voltar a ficar online</t>
+          <t>Trocar de aba sem video aberto</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Refresh recarrega do servidor</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
+          <t>Sem erro ou crash; startAt permanece 0</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1887,17 +1887,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Marcar feito offline</t>
+          <t>Abrir treinos online e depois offline</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Trata erro de rede sem deslogar</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Treinos continuam visiveis (cache)</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Critico</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -1916,17 +1916,17 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Internet lenta / timeout</t>
+          <t>Abrir offline sem cache (1a vez)</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Loading e depois erro tratavel; sem travar</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Mensagem amigavel; sem crash/logout</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Critico</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr"/>
@@ -1935,22 +1935,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Banco Local</t>
+          <t>Offline-First</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>1a execucao (app recem-instalado)</t>
+          <t>Backend desligado</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Cria banco local sem erro; login funciona</t>
+          <t>Erro com Tentar novamente; sem logout</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -1964,27 +1964,27 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Banco Local</t>
+          <t>Offline-First</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Limpar dados do app e reabrir</t>
+          <t>Voltar a ficar online</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Recria tudo; pede login; sem crash</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Critico</t>
+          <t>Refresh recarrega do servidor</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr"/>
@@ -1993,22 +1993,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Banco Local</t>
+          <t>Offline-First</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Reinstalar o app</t>
+          <t>Marcar feito offline</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Sem residuo que quebre a criacao do banco</t>
+          <t>Trata erro de rede sem deslogar</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
@@ -2022,22 +2022,22 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Banco Local</t>
+          <t>Offline-First</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Uso prolongado / muitos treinos</t>
+          <t>Internet lenta / timeout</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Cache nao corrompe nem trava</t>
+          <t>Loading e depois erro tratavel; sem travar</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -2051,27 +2051,27 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>GIA (Chat)</t>
+          <t>Banco Local</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Enviar pergunta</t>
+          <t>1a execucao (app recem-instalado)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Recebe resposta; tela inicial com mascote</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Cria banco local sem erro; login funciona</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Critico</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr"/>
@@ -2080,27 +2080,27 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>GIA (Chat)</t>
+          <t>Banco Local</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Mensagem vazia</t>
+          <t>Limpar dados do app e reabrir</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Nao envia</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Recria tudo; pede login; sem crash</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Critico</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr"/>
@@ -2109,22 +2109,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>GIA (Chat)</t>
+          <t>Banco Local</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Offline / backend fora</t>
+          <t>Reinstalar o app</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Erro tratavel; sem crash/logout</t>
+          <t>Sem residuo que quebre a criacao do banco</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
@@ -2138,27 +2138,27 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>GIA (Chat)</t>
+          <t>Banco Local</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Mensagem longa / caracteres especiais</t>
+          <t>Uso prolongado / muitos treinos</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Sem quebra de layout</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Cache nao corrompe nem trava</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr"/>
@@ -2167,7 +2167,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2177,17 +2177,17 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Enviar varias seguidas</t>
+          <t>Enviar pergunta</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Nao duplica nem trava</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Recebe resposta; tela inicial com mascote</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
@@ -2196,27 +2196,27 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Perfil/Foto</t>
+          <t>GIA (Chat)</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Camera e galeria</t>
+          <t>Mensagem vazia</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Foto aparece; persiste apos reabrir</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Nao envia</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr"/>
@@ -2225,22 +2225,22 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Perfil/Foto</t>
+          <t>GIA (Chat)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Negar permissao de camera</t>
+          <t>Offline / backend fora</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Mensagem amigavel; sem crash</t>
+          <t>Erro tratavel; sem crash/logout</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -2254,22 +2254,22 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Perfil/Foto</t>
+          <t>GIA (Chat)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Foto por usuario</t>
+          <t>Mensagem longa / caracteres especiais</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Foto do A nao aparece para o B</t>
+          <t>Sem quebra de layout</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
@@ -2283,22 +2283,22 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>UI/Tema/Nav</t>
+          <t>GIA (Chat)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Alternar tema claro/escuro</t>
+          <t>Enviar varias seguidas</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Tudo legivel; mascote/icones visiveis</t>
+          <t>Nao duplica nem trava</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
@@ -2312,27 +2312,27 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>UI/Tema/Nav</t>
+          <t>Perfil/Foto</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Tema persiste</t>
+          <t>Camera e galeria</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Reabrir mantem a preferencia</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Foto aparece; persiste apos reabrir</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr"/>
@@ -2341,27 +2341,27 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>UI/Tema/Nav</t>
+          <t>Perfil/Foto</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Navbar (todas as abas)</t>
+          <t>Negar permissao de camera</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Icones do tamanho certo; sem sobreposicao</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Mensagem amigavel; sem crash</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr"/>
@@ -2370,27 +2370,27 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>UI/Tema/Nav</t>
+          <t>Perfil/Foto</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Rotacao / fontes grandes</t>
+          <t>Foto por usuario</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Layout nao estoura (overflow)</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Foto do A nao aparece para o B</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr"/>
@@ -2399,7 +2399,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2409,17 +2409,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Botao voltar do Android</t>
+          <t>Alternar tema claro/escuro</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Navega certo; nao fecha o app sem querer</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Tudo legivel; mascote/icones visiveis</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
@@ -2428,7 +2428,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -2438,17 +2438,17 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Teclado em formularios</t>
+          <t>Tema persiste</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Campos nao ficam escondidos; sem overflow</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Reabrir mantem a preferencia</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr"/>
@@ -2457,27 +2457,27 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Inputs extremos</t>
+          <t>UI/Tema/Nav</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Textos enormes em nome/descricao</t>
+          <t>Navbar (todas as abas)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Trunca/aceita sem corromper</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Icones do tamanho certo; sem sobreposicao</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr"/>
@@ -2486,27 +2486,27 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Inputs extremos</t>
+          <t>UI/Tema/Nav</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Emojis e acentuacao em todos os campos</t>
+          <t>Rotacao / fontes grandes</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Salva e exibe corretamente</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Layout nao estoura (overflow)</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr"/>
@@ -2515,22 +2515,22 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Inputs extremos</t>
+          <t>UI/Tema/Nav</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Numeros negativos/zero/decimais/texto</t>
+          <t>Botao voltar do Android</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Validados; nao quebram a API</t>
+          <t>Navega certo; nao fecha o app sem querer</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -2544,27 +2544,27 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Inputs extremos</t>
+          <t>UI/Tema/Nav</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Espacos em branco / so espacos</t>
+          <t>Teclado em formularios</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Tratados como vazio onde aplicavel</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Campos nao ficam escondidos; sem overflow</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr"/>
@@ -2573,7 +2573,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Duplo clique rapido no salvar</t>
+          <t>Textos enormes em nome/descricao</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Nao duplica; botao desabilita no envio</t>
+          <t>Trunca/aceita sem corromper</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
@@ -2602,22 +2602,22 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>12.1.1</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Visual/Imagens</t>
+          <t>Inputs extremos</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Logo no topo (claro x escuro)</t>
+          <t>Emojis e acentuacao em todos os campos</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Versao certa por tema; nitida</t>
+          <t>Salva e exibe corretamente</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
@@ -2631,22 +2631,22 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>12.1.2</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Visual/Imagens</t>
+          <t>Inputs extremos</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Mascote GIA na tela do chat</t>
+          <t>Numeros negativos/zero/decimais/texto</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Visivel e legivel nos dois temas</t>
+          <t>Validados; nao quebram a API</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
@@ -2660,27 +2660,27 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>12.1.3</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Visual/Imagens</t>
+          <t>Inputs extremos</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Mascote GIA na navbar</t>
+          <t>Espacos em branco / so espacos</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Tamanho dos outros icones; centralizada</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Tratados como vazio onde aplicavel</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr"/>
@@ -2689,27 +2689,27 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>12.1.4</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Visual/Imagens</t>
+          <t>Inputs extremos</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Icone GIA no card do Dashboard</t>
+          <t>Duplo clique rapido no salvar</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Proporcional; sem cortar</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Nao duplica; botao desabilita no envio</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr"/>
@@ -2718,7 +2718,7 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>12.1.5</t>
+          <t>12.1.1</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -2728,17 +2728,17 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Thumbnails de video</t>
+          <t>Logo no topo (claro x escuro)</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Carregam; placeholder; fallback se falhar</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Versao certa por tema; nitida</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr"/>
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>12.1.6</t>
+          <t>12.1.2</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2757,17 +2757,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Foto de perfil</t>
+          <t>Mascote GIA na tela do chat</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Recorte circular; sem esticar</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Visivel e legivel nos dois temas</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr"/>
@@ -2776,7 +2776,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>12.1.7</t>
+          <t>12.1.3</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -2786,17 +2786,17 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Icones em geral</t>
+          <t>Mascote GIA na navbar</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Cor adequada ao tema; nada sumido</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Tamanho dos outros icones; centralizada</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr"/>
@@ -2805,22 +2805,22 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>12.2.1</t>
+          <t>12.1.4</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Visual/Tema</t>
+          <t>Visual/Imagens</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Alternar tema com app aberto</t>
+          <t>Icone GIA no card do Dashboard</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Atualiza na hora, sem reiniciar</t>
+          <t>Proporcional; sem cortar</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr">
@@ -2834,22 +2834,22 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>12.2.2</t>
+          <t>12.1.5</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Visual/Tema</t>
+          <t>Visual/Imagens</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Contraste de textos</t>
+          <t>Thumbnails de video</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Suficiente em todos (nada cinza-sobre-cinza)</t>
+          <t>Carregam; placeholder; fallback se falhar</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
@@ -2863,27 +2863,27 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>12.2.3</t>
+          <t>12.1.6</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Visual/Tema</t>
+          <t>Visual/Imagens</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Campos de formulario</t>
+          <t>Foto de perfil</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Label/hint/borda/erro legiveis nos 2 temas</t>
-        </is>
-      </c>
-      <c r="E82" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Recorte circular; sem esticar</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr"/>
@@ -2892,22 +2892,22 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>12.2.4</t>
+          <t>12.1.7</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Visual/Tema</t>
+          <t>Visual/Imagens</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Cards e divisorias</t>
+          <t>Icones em geral</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Bordas/sombras visiveis sem vazar</t>
+          <t>Cor adequada ao tema; nada sumido</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
@@ -2921,7 +2921,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>12.2.5</t>
+          <t>12.2.1</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2931,12 +2931,12 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Botoes (primario/secundario/perigo)</t>
+          <t>Alternar tema com app aberto</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Cores certas; texto legivel; estado desabilitado</t>
+          <t>Atualiza na hora, sem reiniciar</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
@@ -2950,7 +2950,7 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>12.2.6</t>
+          <t>12.2.2</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
@@ -2960,12 +2960,12 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>SnackBars e dialogos</t>
+          <t>Contraste de textos</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Fundo/texto legiveis nos 2 temas</t>
+          <t>Suficiente em todos (nada cinza-sobre-cinza)</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
@@ -2979,22 +2979,22 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>12.3.1</t>
+          <t>12.2.3</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Visual/Layout</t>
+          <t>Visual/Tema</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Telas pequenas e grandes</t>
+          <t>Campos de formulario</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Sem overflow (faixa listrada)</t>
+          <t>Label/hint/borda/erro legiveis nos 2 temas</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
@@ -3008,27 +3008,27 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>12.3.2</t>
+          <t>12.2.4</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Visual/Layout</t>
+          <t>Visual/Tema</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Fonte grande do sistema</t>
+          <t>Cards e divisorias</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Layout se adapta; texto nao corta</t>
-        </is>
-      </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Bordas/sombras visiveis sem vazar</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr"/>
@@ -3037,27 +3037,27 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>12.3.3</t>
+          <t>12.2.5</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Visual/Layout</t>
+          <t>Visual/Tema</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Rotacao retrato/paisagem</t>
+          <t>Botoes (primario/secundario/perigo)</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Nao quebra nem perde estado</t>
-        </is>
-      </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Cores certas; texto legivel; estado desabilitado</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr"/>
@@ -3066,22 +3066,22 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>12.3.4</t>
+          <t>12.2.6</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Visual/Layout</t>
+          <t>Visual/Tema</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Teclado aberto</t>
+          <t>SnackBars e dialogos</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Campo em foco visivel; nada coberto</t>
+          <t>Fundo/texto legiveis nos 2 temas</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -3095,7 +3095,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>12.3.5</t>
+          <t>12.3.1</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -3105,17 +3105,17 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Textos longos</t>
+          <t>Telas pequenas e grandes</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Quebra ou ellipsis; sem estourar card</t>
-        </is>
-      </c>
-      <c r="E90" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Sem overflow (faixa listrada)</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr"/>
@@ -3124,7 +3124,7 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>12.3.6</t>
+          <t>12.3.2</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Notch/recorte e barra de gestos</t>
+          <t>Fonte grande do sistema</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Conteudo nao fica sob notch/navbar</t>
+          <t>Layout se adapta; texto nao corta</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -3153,7 +3153,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>12.3.7</t>
+          <t>12.3.3</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -3163,17 +3163,17 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Listas longas</t>
+          <t>Rotacao retrato/paisagem</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Rolagem suave; ultimo item nao some atras da navbar/FAB</t>
-        </is>
-      </c>
-      <c r="E92" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Nao quebra nem perde estado</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr"/>
@@ -3182,27 +3182,27 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>12.4.1</t>
+          <t>12.3.4</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Visual/Estados</t>
+          <t>Visual/Layout</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Carregando</t>
+          <t>Teclado aberto</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Spinner centralizado; sem pular layout</t>
-        </is>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Campo em foco visivel; nada coberto</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr"/>
@@ -3211,22 +3211,22 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>12.4.2</t>
+          <t>12.3.5</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Visual/Estados</t>
+          <t>Visual/Layout</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Vazio</t>
+          <t>Textos longos</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Empty state com icone + texto explicativo</t>
+          <t>Quebra ou ellipsis; sem estourar card</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr">
@@ -3240,22 +3240,22 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>12.4.3</t>
+          <t>12.3.6</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Visual/Estados</t>
+          <t>Visual/Layout</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Erro</t>
+          <t>Notch/recorte e barra de gestos</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Mensagem clara + Tentar novamente</t>
+          <t>Conteudo nao fica sob notch/navbar</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
@@ -3269,22 +3269,22 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>12.4.4</t>
+          <t>12.3.7</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Visual/Estados</t>
+          <t>Visual/Layout</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Pull-to-refresh</t>
+          <t>Listas longas</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Indicador aparece e some certo</t>
+          <t>Rolagem suave; ultimo item nao some atras da navbar/FAB</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr">
@@ -3298,22 +3298,22 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>12.5.1</t>
+          <t>12.4.1</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Visual/Consist.</t>
+          <t>Visual/Estados</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Navbar PROF e ALUNO</t>
+          <t>Carregando</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Selecionado destacado; rotulos nao cortados</t>
+          <t>Spinner centralizado; sem pular layout</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr">
@@ -3327,27 +3327,27 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>12.5.2</t>
+          <t>12.4.2</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Visual/Consist.</t>
+          <t>Visual/Estados</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>FAB</t>
+          <t>Vazio</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Nao sobrepoe conteudo; sem crash de Hero</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>Critico</t>
+          <t>Empty state com icone + texto explicativo</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr"/>
@@ -3356,27 +3356,27 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>12.5.3</t>
+          <t>12.4.3</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Visual/Consist.</t>
+          <t>Visual/Estados</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Menu 3 pontos (editar/excluir)</t>
+          <t>Erro</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Abre alinhado; opcoes legiveis</t>
-        </is>
-      </c>
-      <c r="E99" s="6" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Mensagem clara + Tentar novamente</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr"/>
@@ -3385,27 +3385,27 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>12.5.4</t>
+          <t>12.4.4</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Visual/Consist.</t>
+          <t>Visual/Estados</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Botao durante envio</t>
+          <t>Pull-to-refresh</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Vira loading e desabilita</t>
-        </is>
-      </c>
-      <c r="E100" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Indicador aparece e some certo</t>
+        </is>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr"/>
@@ -3414,7 +3414,7 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>12.5.5</t>
+          <t>12.5.1</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
@@ -3424,12 +3424,12 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Selo Concluido / Desmarcar</t>
+          <t>Navbar PROF e ALUNO</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Cores e icones corretos; alinhados</t>
+          <t>Selecionado destacado; rotulos nao cortados</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -3443,7 +3443,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>12.5.6</t>
+          <t>12.5.2</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3453,17 +3453,17 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Espacamentos/alinhamentos</t>
+          <t>FAB</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Padrao consistente entre telas</t>
-        </is>
-      </c>
-      <c r="E102" s="7" t="inlineStr">
-        <is>
-          <t>Baixo</t>
+          <t>Nao sobrepoe conteudo; sem crash de Hero</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>Critico</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr"/>
@@ -3472,31 +3472,147 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>12.6.1</t>
+          <t>12.5.3</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Visual/Varredura</t>
+          <t>Visual/Consist.</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Passar tela a tela (claro+escuro)</t>
+          <t>Menu 3 pontos (editar/excluir)</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Inicial, Login, Cadastro, Dashboard, Treinos, Perfil, GIA, Config, Exercicios, Criar/Editar Treino, Alunos: sem overflow/contraste/imagens/estados</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>Abre alinhado; opcoes legiveis</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
       <c r="F103" s="4" t="inlineStr"/>
       <c r="G103" s="4" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>12.5.4</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Visual/Consist.</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Botao durante envio</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Vira loading e desabilita</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>12.5.5</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Visual/Consist.</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>Selo Concluido / Desmarcar</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Cores e icones corretos; alinhados</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr"/>
+      <c r="G105" s="4" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>12.5.6</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Visual/Consist.</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Espacamentos/alinhamentos</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Padrao consistente entre telas</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>12.6.1</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Visual/Varredura</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Passar tela a tela (claro+escuro)</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>Inicial, Login, Cadastro, Dashboard, Treinos, Perfil, GIA, Config, Exercicios, Criar/Editar Treino, Alunos: sem overflow/contraste/imagens/estados</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G103"/>
@@ -3786,6 +3902,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3793,7 +3910,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
@@ -3803,7 +3920,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -3813,7 +3930,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -3826,6 +3943,7 @@
         <v>15</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>